<commit_message>
Rapport du 22 Aout 2026
</commit_message>
<xml_diff>
--- a/Donnees_Mensuelle.xlsx
+++ b/Donnees_Mensuelle.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84BD8E1-B206-44BD-BCE9-99482BFFF2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713383B5-E5C8-4642-BEBB-4B7497999D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25859,7 +25859,7 @@
     </row>
     <row r="503" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A503" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B503" s="1">
         <v>0</v>
@@ -25908,7 +25908,7 @@
     </row>
     <row r="504" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A504" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B504" s="1">
         <v>0</v>
@@ -25957,7 +25957,7 @@
     </row>
     <row r="505" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A505" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B505" s="1">
         <v>0</v>
@@ -26006,7 +26006,7 @@
     </row>
     <row r="506" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A506" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B506" s="1">
         <v>0</v>
@@ -26055,7 +26055,7 @@
     </row>
     <row r="507" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A507" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B507" s="1">
         <v>0</v>
@@ -26104,7 +26104,7 @@
     </row>
     <row r="508" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A508" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B508" s="1">
         <v>0</v>
@@ -26153,7 +26153,7 @@
     </row>
     <row r="509" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A509" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B509" s="1">
         <v>0</v>
@@ -26202,7 +26202,7 @@
     </row>
     <row r="510" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A510" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B510" s="1">
         <v>0</v>
@@ -26251,7 +26251,7 @@
     </row>
     <row r="511" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A511" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B511" s="1">
         <v>0</v>
@@ -26300,7 +26300,7 @@
     </row>
     <row r="512" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A512" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B512" s="1">
         <v>0</v>
@@ -26349,7 +26349,7 @@
     </row>
     <row r="513" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A513" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B513" s="1">
         <v>0</v>
@@ -26398,7 +26398,7 @@
     </row>
     <row r="514" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A514" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B514" s="1">
         <v>0</v>
@@ -26447,7 +26447,7 @@
     </row>
     <row r="515" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A515" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B515" s="1">
         <v>0</v>
@@ -26496,7 +26496,7 @@
     </row>
     <row r="516" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A516" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B516" s="1">
         <v>0</v>
@@ -26545,7 +26545,7 @@
     </row>
     <row r="517" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A517" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B517" s="1">
         <v>0</v>
@@ -26594,7 +26594,7 @@
     </row>
     <row r="518" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A518" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B518" s="1">
         <v>0</v>
@@ -26643,7 +26643,7 @@
     </row>
     <row r="519" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A519" s="2">
-        <v>46255</v>
+        <v>46254</v>
       </c>
       <c r="B519" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
Rapport du 07 Septembre 2026
</commit_message>
<xml_diff>
--- a/Donnees_Mensuelle.xlsx
+++ b/Donnees_Mensuelle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FC7253-F186-408C-84C8-232E2101A4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D88D5A-8C4C-4971-97E3-A118B7BFFD47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>